<commit_message>
Exclude Simples Nacional from administrative expenses
Removes Simples Nacional from ADM expense totals because it is already
represented by the 9.2% tax applied on sales in the dashboard.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Despesas_RBT_Normalizadas.xlsx
+++ b/Despesas_RBT_Normalizadas.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2047,7 +2047,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2056,12 +2056,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Simples Nacional - Ref. JUN/2026</t>
+          <t>Difal Negociação</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2080,62 +2080,14 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>12460.05</v>
+        <v>1739.18</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Simples Nacional</t>
+          <t>Difal Negociação</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
-        <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Secretaria de Estado de Fazenda de Minas Gerais</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Difal Negociação</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
-      <c r="H36" t="n">
-        <v>1739.18</v>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Difal Negociação</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
         <is>
           <t>SEF/MG</t>
         </is>
@@ -2152,7 +2104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2375,11 +2327,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Simples Nacional</t>
+          <t>Visita cliente</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12460.05</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16">
@@ -2390,25 +2342,10 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Visita cliente</t>
+          <t>Água</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Água</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
         <v>158.19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update administrative expenses from new Despesas_RBT upload
Supports the simplified Fornecedor/Histórico/Valor layout, refreshes
categorization, and regenerates the dashboard excluding Simples Nacional.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Despesas_RBT_Normalizadas.xlsx
+++ b/Despesas_RBT_Normalizadas.xlsx
@@ -483,11 +483,7 @@
           <t>Cesta básica</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -498,11 +494,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>120</v>
       </c>
@@ -528,14 +520,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Salário Jun/26</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -546,11 +534,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>1529</v>
       </c>
@@ -579,11 +563,7 @@
           <t>Vale Transporte Jul/26</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -594,11 +574,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>375.9</v>
       </c>
@@ -624,14 +600,10 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BDMG PRONAMPE 2022 CONTRATO 364182 - PARCELA 23/36</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
+          <t>Empréstimo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -642,11 +614,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>5920.08</v>
       </c>
@@ -672,14 +640,10 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Portal de compra</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
+          <t>Portal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -690,11 +654,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>280.81</v>
       </c>
@@ -723,11 +683,7 @@
           <t>Portal</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -738,11 +694,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>120</v>
       </c>
@@ -771,11 +723,7 @@
           <t>Cesta básica</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -786,11 +734,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>120</v>
       </c>
@@ -816,14 +760,10 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>JUN/26 venc. 06/07</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -834,11 +774,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>2300</v>
       </c>
@@ -864,14 +800,10 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Desinfetante 5L</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
+          <t>Manutenção e limpeza</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -882,11 +814,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>13.99</v>
       </c>
@@ -897,7 +825,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Material/Limpeza</t>
+          <t>Manutenção/Limpeza</t>
         </is>
       </c>
     </row>
@@ -912,14 +840,10 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dias trabalhados 20 a 26 de Julho</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -930,11 +854,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>420</v>
       </c>
@@ -960,14 +880,10 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Energia elétrica</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Energia</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -978,11 +894,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>384.24</v>
       </c>
@@ -1008,14 +920,10 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Água/esgoto</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
+          <t>Água</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1026,11 +934,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>158.19</v>
       </c>
@@ -1070,13 +974,9 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Parcialmente atrasada</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>7000</v>
+        <v>13000</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1100,14 +1000,10 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Visita Cliente</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
+          <t>Despesas comerciais</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1118,11 +1014,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>150</v>
       </c>
@@ -1133,7 +1025,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Visita cliente</t>
+          <t>Despesas comerciais</t>
         </is>
       </c>
     </row>
@@ -1151,11 +1043,7 @@
           <t>Cesta básica</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1166,11 +1054,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>120</v>
       </c>
@@ -1196,14 +1080,10 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Salário Jun/26</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1214,11 +1094,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>1529</v>
       </c>
@@ -1247,11 +1123,7 @@
           <t>Vale transporte Jul/26</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1262,11 +1134,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>262.5</v>
       </c>
@@ -1295,11 +1163,7 @@
           <t>Aluguel Galpão</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1310,11 +1174,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>3454.47</v>
       </c>
@@ -1343,11 +1203,7 @@
           <t>Cesta básica</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1358,11 +1214,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>120</v>
       </c>
@@ -1388,14 +1240,10 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Salário Jun/26</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1406,11 +1254,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>2405</v>
       </c>
@@ -1436,14 +1280,10 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Vale transporte Jul/26 (Não veio11/06 e 17/06)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Vale Transporte Jul/26</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1454,11 +1294,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
         <v>250</v>
       </c>
@@ -1484,14 +1320,10 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Recebimento 1/3 de férias</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
+          <t>Férias</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1502,11 +1334,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>466.67</v>
       </c>
@@ -1532,14 +1360,10 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JUN/26 venc. 06/07</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1550,11 +1374,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
         <v>1730</v>
       </c>
@@ -1580,14 +1400,10 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Devolução do celular via Correios</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+          <t>Frete</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1598,11 +1414,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
         <v>34</v>
       </c>
@@ -1613,7 +1425,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Despesas diversas</t>
+          <t>Frete/Diversos</t>
         </is>
       </c>
     </row>
@@ -1631,11 +1443,7 @@
           <t>Rescisão</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1646,11 +1454,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
         <v>4723</v>
       </c>
@@ -1679,11 +1483,7 @@
           <t>Honorário Contabilidade</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1694,11 +1494,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>864.76</v>
       </c>
@@ -1727,11 +1523,7 @@
           <t>Honorários Contábeis - Venda 1889</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1742,11 +1534,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
         <v>923.48</v>
       </c>
@@ -1772,14 +1560,10 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FGTS - RESCISORIA MAIRA</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+          <t>FGTS</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1790,11 +1574,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
         <v>951.39</v>
       </c>
@@ -1820,14 +1600,10 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FGTS - 06/2026</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
+          <t>FGTS</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1838,11 +1614,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
         <v>707.2</v>
       </c>
@@ -1868,14 +1640,10 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GUIA DCTFWEB 06/2026</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
+          <t>Difal Negociação</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1886,22 +1654,18 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
         <v>768.46</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Pessoal</t>
+          <t>Difal Negociação</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Encargos sociais (INSS/FGTS)</t>
+          <t>SEF/MG</t>
         </is>
       </c>
     </row>
@@ -1930,13 +1694,9 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Parcialmente atrasada</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>7000</v>
+        <v>13000</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1963,11 +1723,7 @@
           <t>Empréstimo</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -1978,11 +1734,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
         <v>1205</v>
       </c>
@@ -2011,11 +1763,7 @@
           <t>Difal Antecipação</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -2026,11 +1774,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
         <v>2230.27</v>
       </c>
@@ -2059,11 +1803,7 @@
           <t>Difal Negociação</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -2074,11 +1814,7 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
         <v>1739.18</v>
       </c>
@@ -2196,7 +1932,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1739.18</v>
+        <v>2507.64</v>
       </c>
     </row>
     <row r="7">
@@ -2286,7 +2022,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18898.12</v>
+        <v>18129.66</v>
       </c>
     </row>
     <row r="13">
@@ -2316,7 +2052,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14000</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Inclui comissão de vendas (R$ 2.500) nas despesas de julho
Atualiza FGTS (R$ 804,54) conforme planilha enviada e regenera o dashboard.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Despesas_RBT_Normalizadas.xlsx
+++ b/Despesas_RBT_Normalizadas.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>951.39</v>
+        <v>804.54</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1826,6 +1826,46 @@
       <c r="J35" t="inlineStr">
         <is>
           <t>SEF/MG</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Vendedor 1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Comissão de Vendas</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Comissão de vendas</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Comissão de vendas</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1898,11 +1938,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Contabilidade</t>
+          <t>Comissão de vendas</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1788.24</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="5">
@@ -1913,11 +1953,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Difal Antecipação</t>
+          <t>Contabilidade</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2230.27</v>
+        <v>1788.24</v>
       </c>
     </row>
     <row r="6">
@@ -1928,11 +1968,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Difal Negociação</t>
+          <t>Difal Antecipação</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2507.64</v>
+        <v>2230.27</v>
       </c>
     </row>
     <row r="7">
@@ -1943,11 +1983,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Empréstimo Rosa Amasiles</t>
+          <t>Difal Negociação</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1205</v>
+        <v>2507.64</v>
       </c>
     </row>
     <row r="8">
@@ -1958,11 +1998,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Internet/Sistemas</t>
+          <t>Empréstimo Rosa Amasiles</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>120</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="9">
@@ -1973,11 +2013,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Luz</t>
+          <t>Internet/Sistemas</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>384.24</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -1988,11 +2028,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Manutenção e reparos</t>
+          <t>Luz</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13.99</v>
+        <v>384.24</v>
       </c>
     </row>
     <row r="11">
@@ -2003,11 +2043,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Manutenção e reparos</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>34</v>
+        <v>13.99</v>
       </c>
     </row>
     <row r="12">
@@ -2018,11 +2058,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pessoal</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18129.66</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
@@ -2033,11 +2073,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Portal de compra</t>
+          <t>Pessoal</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>280.81</v>
+        <v>17982.81</v>
       </c>
     </row>
     <row r="14">
@@ -2048,11 +2088,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pró-labore</t>
+          <t>Portal de compra</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>26000</v>
+        <v>280.81</v>
       </c>
     </row>
     <row r="15">
@@ -2063,11 +2103,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Visita cliente</t>
+          <t>Pró-labore</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>150</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="16">
@@ -2078,10 +2118,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Visita cliente</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Água</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>158.19</v>
       </c>
     </row>

</xml_diff>